<commit_message>
Fix live baseline deployment package
</commit_message>
<xml_diff>
--- a/runtime_outputs/DAILY_MARKET_RECORD.xlsx
+++ b/runtime_outputs/DAILY_MARKET_RECORD.xlsx
@@ -14,19 +14,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current_Prices" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current_Holdings" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Report" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_Price_Refresh" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auto_Rebalance" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target_Price_Refresh" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Today_Order_Plan'!$A$1:$AG$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Order_History'!$A$1:$W$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market_State'!$A$1:$AI$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Target_Position'!$A$1:$K$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Current_Prices'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Today_Order_Plan'!$A$1:$AI$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Order_History'!$A$1:$W$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market_State'!$A$1:$AM$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Target_Position'!$A$1:$K$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Current_Prices'!$A$1:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Current_Holdings'!$A$1:$A$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Update_Report'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Summary'!$A$1:$AG$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Target_Price_Refresh'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Update_Report'!$A$1:$P$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Auto_Rebalance'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Summary'!$A$1:$AG$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Target_Price_Refresh'!$A$1:$P$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,14 +445,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG8"/>
+  <dimension ref="A1:AI7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
@@ -458,27 +460,29 @@
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
-    <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="19" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="19" customWidth="1" min="24" max="24"/>
-    <col width="21" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="19" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="21" customWidth="1" min="28" max="28"/>
-    <col width="21" customWidth="1" min="29" max="29"/>
-    <col width="17" customWidth="1" min="30" max="30"/>
-    <col width="20" customWidth="1" min="31" max="31"/>
-    <col width="23" customWidth="1" min="32" max="32"/>
+    <col width="21" customWidth="1" min="27" max="27"/>
+    <col width="19" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="31" max="31"/>
+    <col width="17" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="23" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,105 +548,115 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>current_price_date</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>current_price_source</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>target_amount</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>target_shares</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>current_shares</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>diff_shares</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>entry_status</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>entry_gap_pct</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>entry_current_price</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>entry_signal_date</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>entry_signal_close</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>buy_lower_price</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>buy_upper_price</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>partial_upper_price</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>hard_upper_price</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>tracking_base_date</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>tracking_base_price</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>tracking_return_pct</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>entry_floor_pct</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>entry_full_cap_pct</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>entry_partial_cap_pct</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>entry_hard_cap_pct</t>
         </is>
@@ -656,12 +670,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2327.TW</t>
+          <t>2492.TW</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>國巨*</t>
+          <t>華新科</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -670,93 +684,103 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="F2" t="n">
-        <v>940</v>
+        <v>561</v>
       </c>
       <c r="G2" t="n">
-        <v>1080</v>
+        <v>561</v>
       </c>
       <c r="H2" t="n">
-        <v>1080</v>
+        <v>561</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="M2" t="n">
-        <v>333333.3333333333</v>
-      </c>
-      <c r="N2" t="n">
-        <v>308</v>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="P2" t="n">
-        <v>308</v>
-      </c>
-      <c r="Q2" t="inlineStr">
+        <v>891</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>891</v>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>禁止新買</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>28.26603325415677</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1080</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>842</v>
-      </c>
-      <c r="W2" t="n">
-        <v>783.0599999999999</v>
+        <v>561</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="X2" t="n">
-        <v>867.26</v>
+        <v>561</v>
       </c>
       <c r="Y2" t="n">
-        <v>867.26</v>
+        <v>521.73</v>
       </c>
       <c r="Z2" t="n">
-        <v>867.26</v>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+        <v>577.83</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>577.83</v>
       </c>
       <c r="AB2" t="n">
-        <v>842</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>28.26603325415677</v>
+        <v>577.83</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="AD2" t="n">
+        <v>561</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
         <v>-7</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>3</v>
       </c>
       <c r="AG2" t="n">
         <v>3</v>
       </c>
+      <c r="AH2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -766,216 +790,236 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2454.TW</t>
+          <t>2327.TW</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>國巨*</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ic_design_mobile</t>
+          <t>passive_component</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="F3" t="n">
-        <v>4470</v>
+        <v>1080</v>
       </c>
       <c r="G3" t="n">
-        <v>4390</v>
+        <v>1080</v>
       </c>
       <c r="H3" t="n">
-        <v>4390</v>
+        <v>1080</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="M3" t="n">
-        <v>333333.3333333333</v>
-      </c>
-      <c r="N3" t="n">
-        <v>75</v>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="P3" t="n">
-        <v>75</v>
-      </c>
-      <c r="Q3" t="inlineStr">
+        <v>462</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>462</v>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>禁止新買</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>7.466340269277838</v>
-      </c>
-      <c r="T3" t="n">
-        <v>4390</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>4085</v>
-      </c>
-      <c r="W3" t="n">
-        <v>3799.05</v>
+        <v>1080</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="X3" t="n">
-        <v>4207.55</v>
+        <v>1080</v>
       </c>
       <c r="Y3" t="n">
-        <v>4207.55</v>
+        <v>1004.4</v>
       </c>
       <c r="Z3" t="n">
-        <v>4207.55</v>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+        <v>1112.4</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1112.4</v>
       </c>
       <c r="AB3" t="n">
-        <v>4085</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>7.466340269277838</v>
+        <v>1112.4</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="AD3" t="n">
+        <v>1080</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="n">
         <v>-7</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>3</v>
       </c>
       <c r="AG3" t="n">
         <v>3</v>
       </c>
+      <c r="AH3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3189.TW</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>Sandisk Corporation - Common Stock When-Issued</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>substrate</t>
+          <t>memory_storage</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.25</v>
       </c>
       <c r="F4" t="n">
-        <v>660</v>
+        <v>2184.75</v>
       </c>
       <c r="G4" t="n">
-        <v>724</v>
+        <v>2184.75</v>
       </c>
       <c r="H4" t="n">
-        <v>724</v>
+        <v>2184.75</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="M4" t="n">
-        <v>333333.3333333333</v>
-      </c>
-      <c r="N4" t="n">
-        <v>460</v>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="P4" t="n">
-        <v>460</v>
-      </c>
-      <c r="Q4" t="inlineStr">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>禁止新買</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>16.96284329563813</v>
-      </c>
-      <c r="T4" t="n">
-        <v>724</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>619</v>
-      </c>
-      <c r="W4" t="n">
-        <v>575.67</v>
+        <v>2184.75</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="X4" t="n">
-        <v>637.5700000000001</v>
+        <v>2184.75</v>
       </c>
       <c r="Y4" t="n">
-        <v>637.5700000000001</v>
+        <v>2075.5125</v>
       </c>
       <c r="Z4" t="n">
-        <v>637.5700000000001</v>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+        <v>2293.9875</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>2293.9875</v>
       </c>
       <c r="AB4" t="n">
-        <v>619</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>16.96284329563813</v>
+        <v>2293.9875</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="AD4" t="n">
-        <v>-7</v>
+        <v>2184.75</v>
       </c>
       <c r="AE4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>3</v>
+        <v>-5</v>
       </c>
       <c r="AG4" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -986,107 +1030,117 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sandisk Corporation - Common Stock When-Issued</t>
+          <t>Arm Holdings plc - American Depositary Shares</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>memory_storage</t>
+          <t>ai_compute</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>0.25</v>
       </c>
       <c r="F5" t="n">
-        <v>2184.75</v>
+        <v>439.4599914550781</v>
       </c>
       <c r="G5" t="n">
-        <v>2184.75</v>
+        <v>439.4599914550781</v>
       </c>
       <c r="H5" t="n">
-        <v>2184.75</v>
+        <v>439.4599914550781</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
         <v>25000</v>
       </c>
-      <c r="N5" t="n">
-        <v>11.44295686005264</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
       <c r="P5" t="n">
-        <v>11.44295686005264</v>
-      </c>
-      <c r="Q5" t="inlineStr">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="S5" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>禁止新買</t>
-        </is>
-      </c>
-      <c r="S5" t="n">
-        <v>37.41085075626567</v>
-      </c>
-      <c r="T5" t="n">
-        <v>2184.75</v>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>1589.93994140625</v>
-      </c>
-      <c r="W5" t="n">
-        <v>1510.442944335938</v>
+        <v>439.4599914550781</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="X5" t="n">
-        <v>1669.436938476562</v>
+        <v>439.4599914550781</v>
       </c>
       <c r="Y5" t="n">
-        <v>1669.436938476562</v>
+        <v>417.4869918823242</v>
       </c>
       <c r="Z5" t="n">
-        <v>1669.436938476562</v>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
+        <v>461.432991027832</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>461.432991027832</v>
       </c>
       <c r="AB5" t="n">
-        <v>1589.93994140625</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>37.41085075626567</v>
+        <v>461.432991027832</v>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="AD5" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="n">
         <v>-5</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>5</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>5</v>
       </c>
       <c r="AG5" t="n">
         <v>5</v>
       </c>
+      <c r="AH5" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1096,12 +1150,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Arm Holdings plc - American Depositary Shares</t>
+          <t>Marvell Technology, Inc. - Common Stock</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1113,90 +1167,100 @@
         <v>0.25</v>
       </c>
       <c r="F6" t="n">
-        <v>439.4599914550781</v>
+        <v>310.5799865722656</v>
       </c>
       <c r="G6" t="n">
-        <v>439.4599914550781</v>
+        <v>310.5799865722656</v>
       </c>
       <c r="H6" t="n">
-        <v>439.4599914550781</v>
+        <v>310.5799865722656</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
         <v>25000</v>
       </c>
-      <c r="N6" t="n">
-        <v>56.88800001388867</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
       <c r="P6" t="n">
-        <v>56.88800001388867</v>
-      </c>
-      <c r="Q6" t="inlineStr">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>可買滿</t>
         </is>
       </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" t="n">
-        <v>439.4599914550781</v>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
+      <c r="U6" t="n">
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>439.4599914550781</v>
-      </c>
-      <c r="W6" t="n">
-        <v>417.4869918823242</v>
+        <v>310.5799865722656</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="X6" t="n">
-        <v>461.432991027832</v>
+        <v>310.5799865722656</v>
       </c>
       <c r="Y6" t="n">
-        <v>461.432991027832</v>
+        <v>295.0509872436523</v>
       </c>
       <c r="Z6" t="n">
-        <v>461.432991027832</v>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
+        <v>326.1089859008789</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>326.1089859008789</v>
       </c>
       <c r="AB6" t="n">
-        <v>439.4599914550781</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>0</v>
+        <v>326.1089859008789</v>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="AD6" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
         <v>-5</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>5</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>5</v>
       </c>
       <c r="AG6" t="n">
         <v>5</v>
       </c>
+      <c r="AH6" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1206,220 +1270,299 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Marvell Technology, Inc. - Common Stock</t>
+          <t>Western Digital Corporation - Common Stock</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ai_compute</t>
+          <t>memory_storage</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>0.25</v>
       </c>
       <c r="F7" t="n">
-        <v>310.5799865722656</v>
+        <v>746.22998046875</v>
       </c>
       <c r="G7" t="n">
-        <v>310.5799865722656</v>
+        <v>746.22998046875</v>
       </c>
       <c r="H7" t="n">
-        <v>310.5799865722656</v>
+        <v>746.22998046875</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
         <v>25000</v>
       </c>
-      <c r="N7" t="n">
-        <v>80.49456204797346</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
       <c r="P7" t="n">
-        <v>80.49456204797346</v>
-      </c>
-      <c r="Q7" t="inlineStr">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="S7" t="inlineStr">
         <is>
           <t>新增</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>可買滿</t>
         </is>
       </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>310.5799865722656</v>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
+      <c r="U7" t="n">
+        <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>310.5799865722656</v>
-      </c>
-      <c r="W7" t="n">
-        <v>295.0509872436523</v>
+        <v>746.22998046875</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="X7" t="n">
-        <v>326.1089859008789</v>
+        <v>746.22998046875</v>
       </c>
       <c r="Y7" t="n">
-        <v>326.1089859008789</v>
+        <v>708.9184814453125</v>
       </c>
       <c r="Z7" t="n">
-        <v>326.1089859008789</v>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
+        <v>783.5414794921875</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>783.5414794921875</v>
       </c>
       <c r="AB7" t="n">
-        <v>310.5799865722656</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0</v>
+        <v>783.5414794921875</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="AD7" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
         <v>-5</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>5</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>5</v>
       </c>
       <c r="AG7" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>WDC</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Western Digital Corporation - Common Stock</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>memory_storage</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F8" t="n">
-        <v>746.22998046875</v>
-      </c>
-      <c r="G8" t="n">
-        <v>746.22998046875</v>
-      </c>
-      <c r="H8" t="n">
-        <v>746.22998046875</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>25000</v>
-      </c>
-      <c r="N8" t="n">
-        <v>33.50173626674187</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>33.50173626674187</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>新增</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>可買滿</t>
-        </is>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>746.22998046875</v>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="V8" t="n">
-        <v>746.22998046875</v>
-      </c>
-      <c r="W8" t="n">
-        <v>708.9184814453125</v>
-      </c>
-      <c r="X8" t="n">
-        <v>783.5414794921875</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>783.5414794921875</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>783.5414794921875</v>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="AB8" t="n">
-        <v>746.22998046875</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>-5</v>
-      </c>
-      <c r="AE8" t="n">
+      <c r="AH7" t="n">
         <v>5</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AI7" t="n">
         <v>5</v>
       </c>
-      <c r="AG8" t="n">
-        <v>5</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG8"/>
+  <autoFilter ref="A1:AI7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>finished_at</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>lookback_days</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>chunk_size</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>sleep_seconds</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>timeout</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>retry_attempts</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>retry_sleep_seconds</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>updated_symbols</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>updated_symbol_count</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>current_price_rows</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>markets</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>yfinance_target_only</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:16</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>30</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>['TW:2327.TW', 'TW:2492.TW', 'US:ARM', 'US:MRVL', 'US:SNDK', 'US:WDC']</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N2" t="n">
+        <v>9</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>[{'market': 'TW', 'status': 'updated', 'start': '2026-05-31', 'symbols': ['2327.TW', '2492.TW'], 'attempted_symbols': 2, 'chunks_attempted': 2, 'download_attempts': 2, 'retry_attempts': 2, 'retry_sleep_seconds': 12.0, 'updated_symbols': 2, 'skipped_older': [], 'errors': []}, {'market': 'US', 'status': 'updated', 'start': '2026-05-31', 'symbols': ['ARM', 'MRVL', 'SNDK', 'WDC'], 'attempted_symbols': 4, 'chunks_attempted': 4, 'download_attempts': 4, 'retry_attempts': 2, 'retry_sleep_seconds': 12.0, 'updated_symbols': 4, 'skipped_older': [], 'errors': []}]</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Target-only quote refresh updates state/current_prices.csv and entry judgment only. It does not update the full scan pool or retrain strategy rules.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1430,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W29"/>
+  <dimension ref="A1:W41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -4179,8 +4322,1124 @@
         <v>0</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:15:31</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:49</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2303.TW</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>聯電</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3436</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>3436</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>145.5</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R30" t="n">
+        <v>145.5</v>
+      </c>
+      <c r="S30" t="n">
+        <v>135.315</v>
+      </c>
+      <c r="T30" t="n">
+        <v>149.865</v>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>145.5</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:15:31</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:49</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2327.TW</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>國巨*</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>passive_component</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J31" t="n">
+        <v>462</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>462</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1080</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R31" t="n">
+        <v>1080</v>
+      </c>
+      <c r="S31" t="n">
+        <v>1004.4</v>
+      </c>
+      <c r="T31" t="n">
+        <v>1112.4</v>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>1080</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:15:31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:49</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sandisk Corporation - Common Stock When-Issued</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>memory_storage</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J32" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="S32" t="n">
+        <v>2075.5125</v>
+      </c>
+      <c r="T32" t="n">
+        <v>2293.9875</v>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:15:31</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:49</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Arm Holdings plc - American Depositary Shares</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ai_compute</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J33" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R33" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="S33" t="n">
+        <v>417.4869918823242</v>
+      </c>
+      <c r="T33" t="n">
+        <v>461.432991027832</v>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:15:31</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:49</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Marvell Technology, Inc. - Common Stock</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>ai_compute</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J34" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="S34" t="n">
+        <v>295.0509872436523</v>
+      </c>
+      <c r="T34" t="n">
+        <v>326.1089859008789</v>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="W34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:15:31</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:49</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Western Digital Corporation - Common Stock</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>memory_storage</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J35" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="S35" t="n">
+        <v>708.9184814453125</v>
+      </c>
+      <c r="T35" t="n">
+        <v>783.5414794921875</v>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:26</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2492.TW</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>華新科</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>passive_component</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J36" t="n">
+        <v>891</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>891</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>561</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R36" t="n">
+        <v>561</v>
+      </c>
+      <c r="S36" t="n">
+        <v>521.73</v>
+      </c>
+      <c r="T36" t="n">
+        <v>577.83</v>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V36" t="n">
+        <v>561</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:26</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2327.TW</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>國巨*</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>passive_component</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J37" t="n">
+        <v>462</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>462</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1080</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>1080</v>
+      </c>
+      <c r="S37" t="n">
+        <v>1004.4</v>
+      </c>
+      <c r="T37" t="n">
+        <v>1112.4</v>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V37" t="n">
+        <v>1080</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:26</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sandisk Corporation - Common Stock When-Issued</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>memory_storage</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J38" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R38" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="S38" t="n">
+        <v>2075.5125</v>
+      </c>
+      <c r="T38" t="n">
+        <v>2293.9875</v>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:26</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Arm Holdings plc - American Depositary Shares</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ai_compute</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J39" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R39" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="S39" t="n">
+        <v>417.4869918823242</v>
+      </c>
+      <c r="T39" t="n">
+        <v>461.432991027832</v>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V39" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:26</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Marvell Technology, Inc. - Common Stock</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>ai_compute</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J40" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R40" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="S40" t="n">
+        <v>295.0509872436523</v>
+      </c>
+      <c r="T40" t="n">
+        <v>326.1089859008789</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V40" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="W40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:26</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Western Digital Corporation - Common Stock</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>memory_storage</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J41" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R41" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="S41" t="n">
+        <v>708.9184814453125</v>
+      </c>
+      <c r="T41" t="n">
+        <v>783.5414794921875</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V41" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="W41" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W29"/>
+  <autoFilter ref="A1:W41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4191,16 +5450,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI4"/>
+  <dimension ref="A1:AM4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -4214,21 +5473,25 @@
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="32" customWidth="1" min="19" max="19"/>
     <col width="39" customWidth="1" min="20" max="20"/>
-    <col width="32" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="23" customWidth="1" min="21" max="21"/>
+    <col width="24" customWidth="1" min="22" max="22"/>
     <col width="44" customWidth="1" min="23" max="23"/>
-    <col width="17" customWidth="1" min="24" max="24"/>
-    <col width="10" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="23" customWidth="1" min="27" max="27"/>
-    <col width="44" customWidth="1" min="28" max="28"/>
-    <col width="27" customWidth="1" min="29" max="29"/>
+    <col width="35" customWidth="1" min="24" max="24"/>
+    <col width="27" customWidth="1" min="25" max="25"/>
+    <col width="31" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
     <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="16" customWidth="1" min="31" max="31"/>
-    <col width="34" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="31" customWidth="1" min="34" max="34"/>
-    <col width="31" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="31" max="31"/>
+    <col width="44" customWidth="1" min="32" max="32"/>
+    <col width="27" customWidth="1" min="33" max="33"/>
+    <col width="11" customWidth="1" min="34" max="34"/>
+    <col width="16" customWidth="1" min="35" max="35"/>
+    <col width="34" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="31" customWidth="1" min="38" max="38"/>
+    <col width="31" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4349,60 +5612,80 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
+          <t>research_component_rebalance_date</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>live_cycle_rebalance_date</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>live_cycle_source_signal_date</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>live_cycle_baseline_type</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>execution_top_n</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>regime</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>gross_cap</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>scan_universe_symbols</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>dynamic_market_pool</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>uses_2025_2026_for_tuning</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>top_stock</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>top_theme</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>outside_execution_count_in_top20</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>watch_only</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>feeds_dynamic_market_strategy</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>feeds_dynamic_formal_strategy</t>
         </is>
@@ -4416,17 +5699,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:21</t>
+          <t>2026-06-21T22:54:52</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TWSWENS-002469_TOP1_STRATEGY_SWITCH</t>
+          <t>TW_TOP2_HOLD46_CLEAN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4436,12 +5719,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>top1_strategy_switch</t>
+          <t>top2_h46_strategy_switch</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DEFENSE_040838</t>
+          <t>VALMAX_046612</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -4452,38 +5735,38 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>top1_switch</t>
+          <t>top2_h46_switch</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>DEFENSE_040838</t>
+          <t>VALMAX_046612</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>1.036762904097156</v>
+        <v>0.5977795397936401</v>
       </c>
       <c r="O2" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="S2" t="b">
         <v>0</v>
@@ -4493,17 +5776,37 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>execution_date_not_signal_date</t>
+          <t>live_go_live_cycle</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>hold_top1_target</t>
+          <t>hold_live_cycle_target</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>TW production target uses clean Top1 strategy switch, then applies execution overlay: equal weight across selected stocks. No retraining in cloud package.</t>
+          <t>TW production target uses clean Top2/H46 strategy switch, then applies execution overlay: equal weight across selected stocks. Manual go-live baseline recomputes the initial live target from that baseline close and then holds it until the next live cycle. No retraining in cloud package. Live cycle starts from 2026-06-18 because formal deployment was reset manually.</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>manual_go_live_close</t>
         </is>
       </c>
     </row>
@@ -4520,7 +5823,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:24</t>
+          <t>2026-06-21T22:54:57</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4550,7 +5853,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -4560,47 +5863,67 @@
         <v>10</v>
       </c>
       <c r="P3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
+        <v>10</v>
+      </c>
+      <c r="S3" t="b">
+        <v>0</v>
+      </c>
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>live_go_live_cycle</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>US production target uses the clean dynamic-market switch with Top4 execution and 25% single-stock cap. Rules are frozen; no cloud retraining. Live cycle starts from 2026-06-18 because formal deployment was reset manually.</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>manual_go_live_close</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
         <v>4</v>
       </c>
-      <c r="S3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" t="b">
-        <v>0</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>latest_backtest_step_counter</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>US production target uses the clean dynamic-market switch with Top4 execution and 25% single-stock cap. Rules are frozen; no cloud retraining.</t>
-        </is>
-      </c>
-      <c r="X3" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>risk_on</t>
         </is>
       </c>
-      <c r="Z3" t="n">
+      <c r="AD3" t="n">
         <v>1</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AE3" t="n">
         <v>812</v>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>rolling Top800 by 60D median dollar volume</t>
         </is>
       </c>
-      <c r="AC3" t="b">
+      <c r="AG3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4617,37 +5940,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:26</t>
-        </is>
-      </c>
-      <c r="AA4" t="n">
+          <t>2026-06-21T22:54:59</t>
+        </is>
+      </c>
+      <c r="AE4" t="n">
         <v>812</v>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>memory_storage</t>
         </is>
       </c>
-      <c r="AF4" t="n">
+      <c r="AJ4" t="n">
         <v>11</v>
       </c>
-      <c r="AG4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH4" t="b">
+      <c r="AK4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="b">
         <v>1</v>
       </c>
-      <c r="AI4" t="b">
+      <c r="AM4" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AI4"/>
+  <autoFilter ref="A1:AM4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4658,15 +5981,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="39" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -4739,12 +6062,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2327.TW</t>
+          <t>2492.TW</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>國巨*</t>
+          <t>華新科</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -4754,18 +6077,18 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>top1_DEFENSE_040838|equal_weight_exec</t>
+          <t>top2_h46_VALMAX_046612|equal_weight_exec</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DEFENSE_040838</t>
+          <t>VALMAX_046612</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4787,33 +6110,33 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2454.TW</t>
+          <t>2327.TW</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>國巨*</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ic_design_mobile</t>
+          <t>passive_component</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>top1_DEFENSE_040838|equal_weight_exec</t>
+          <t>top2_h46_VALMAX_046612|equal_weight_exec</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="G3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DEFENSE_040838</t>
+          <t>VALMAX_046612</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4830,49 +6153,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3189.TW</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>Sandisk Corporation - Common Stock When-Issued</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>substrate</t>
+          <t>memory_storage</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>top1_DEFENSE_040838|equal_weight_exec</t>
+          <t>top4_TOP5_R800_N5_COMBO</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DEFENSE_040838</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>TW_EQUAL_WEIGHT</t>
-        </is>
+          <t>TOP5_R800_N5_COMBO</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>3.606551498953182</v>
       </c>
     </row>
     <row r="5">
@@ -4883,17 +6196,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sandisk Corporation - Common Stock When-Issued</t>
+          <t>Arm Holdings plc - American Depositary Shares</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>memory_storage</t>
+          <t>ai_compute</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4910,7 +6223,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>3.606551498953182</v>
+        <v>1.865391188378607</v>
       </c>
     </row>
     <row r="6">
@@ -4921,12 +6234,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Arm Holdings plc - American Depositary Shares</t>
+          <t>Marvell Technology, Inc. - Common Stock</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4948,7 +6261,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>1.865391188378607</v>
+        <v>1.797469120222876</v>
       </c>
     </row>
     <row r="7">
@@ -4959,17 +6272,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Marvell Technology, Inc. - Common Stock</t>
+          <t>Western Digital Corporation - Common Stock</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ai_compute</t>
+          <t>memory_storage</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4986,49 +6299,11 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>1.797469120222876</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>WDC</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Western Digital Corporation - Common Stock</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>memory_storage</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>top4_TOP5_R800_N5_COMBO</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>TOP5_R800_N5_COMBO</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
         <v>1.714474087202342</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K8"/>
+  <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5039,7 +6314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5108,7 +6383,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:34</t>
+          <t>2026-06-21T22:55:10</t>
         </is>
       </c>
     </row>
@@ -5138,7 +6413,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:35</t>
+          <t>2026-06-21T22:55:12</t>
         </is>
       </c>
     </row>
@@ -5168,7 +6443,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:36</t>
+          <t>2026-06-21T22:55:14</t>
         </is>
       </c>
     </row>
@@ -5198,7 +6473,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:37</t>
+          <t>2026-06-21T22:55:16</t>
         </is>
       </c>
     </row>
@@ -5228,7 +6503,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:30</t>
+          <t>2026-06-21T22:55:05</t>
         </is>
       </c>
     </row>
@@ -5292,8 +6567,68 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2303.TW</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>145.5</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-06-21T20:16:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2492.TW</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>561</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>yfinance_target_daily</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:55:07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F8"/>
+  <autoFilter ref="A1:F10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5336,14 +6671,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5359,34 +6705,531 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>new_rows_total</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>source_rate_limited</t>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>new_rows</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>attempted_symbols</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>updated_symbols</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>error_count</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>before_rows</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>before_symbols</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>before_max_date</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>after_rows</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>after_symbols</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>after_max_date</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>path</t>
         </is>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:45:54</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:46:07</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>skipped_full_market_update_target_only_mode</t>
+          <t>US_EXECUTION</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>skipped_preflight_no_new_market_date</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>39891</v>
+      </c>
+      <c r="K2" t="n">
+        <v>95</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>39891</v>
+      </c>
+      <c r="N2" t="n">
+        <v>95</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\01_LOCAL_RUN_REQUIRED\CLOUD_DAILY_MARKET_POOL\data_live\us_execution_prices_tail.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:45:54</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:46:07</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>US_SCAN</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>skipped_daily_safe_mode</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>336937</v>
+      </c>
+      <c r="K3" t="n">
+        <v>812</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>336937</v>
+      </c>
+      <c r="N3" t="n">
+        <v>812</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\01_LOCAL_RUN_REQUIRED\CLOUD_DAILY_MARKET_POOL\data_live\us_scan_prices_tail.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:45:54</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:46:07</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TW_STOCKS</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>skipped_daily_safe_mode</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>817051</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1964</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>817051</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1964</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\01_LOCAL_RUN_REQUIRED\CLOUD_DAILY_MARKET_POOL\data_live\tw_strategy_prices_tail.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:45:54</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-21T22:46:07</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TW_INDEX</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>skipped_preflight_no_new_market_date</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>420</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>420</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\01_LOCAL_RUN_REQUIRED\CLOUD_DAILY_MARKET_POOL\data_live\tw_index_prices_tail.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>started_at</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>finished_at</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>due_markets</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>full_markets</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>decision_text</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>due</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>days_since_rebalance</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rebalance_step</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>quote_date</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>component_rebalance_date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-20T16:59:36</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-20T17:00:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>not_due_fast_update_only</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>V1046 自動換倉判斷
+時間: 2026-06-20T17:00:00
+狀態: not_due_fast_update_only
+換倉到期: 無
+動作: 只更新目前推薦/持倉價格、Dashboard、Excel，不抓全市場。
+換倉週期
+- TW: 3/5 交易日，未到期，價格日 2026-06-20
+- US: 7/10 交易日，未到期，價格日 2026-06-20
+目前正式目標持倉
+- TW: 2327.TW 33.33% 禁止新買 / 2454.TW 33.33% 可買滿 / 4958.TW 33.33% 禁止新買
+- US: SNDK 25.0% 禁止新買 / ARM 25.0% 禁止新買 / MRVL 25.0% 禁止新買 / WDC 25.0% 禁止新買
+JSON報告: D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\CLOUD_DAILY_MARKET_POOL\runtime_outputs\LATEST_AUTO_REBALANCE_REPORT.json
+文字報告: D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\CLOUD_DAILY_MARKET_POOL\runtime_outputs\LATEST_AUTO_REBALANCE_DECISION.txt</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-20T16:59:36</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-20T17:00:00</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>not_due_fast_update_only</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>V1046 自動換倉判斷
+時間: 2026-06-20T17:00:00
+狀態: not_due_fast_update_only
+換倉到期: 無
+動作: 只更新目前推薦/持倉價格、Dashboard、Excel，不抓全市場。
+換倉週期
+- TW: 3/5 交易日，未到期，價格日 2026-06-20
+- US: 7/10 交易日，未到期，價格日 2026-06-20
+目前正式目標持倉
+- TW: 2327.TW 33.33% 禁止新買 / 2454.TW 33.33% 可買滿 / 4958.TW 33.33% 禁止新買
+- US: SNDK 25.0% 禁止新買 / ARM 25.0% 禁止新買 / MRVL 25.0% 禁止新買 / WDC 25.0% 禁止新買
+JSON報告: D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\CLOUD_DAILY_MARKET_POOL\runtime_outputs\LATEST_AUTO_REBALANCE_REPORT.json
+文字報告: D:\V1046_FULL_MARKET_STRATEGY_DATA_PACK\CLOUD_DAILY_MARKET_POOL\runtime_outputs\LATEST_AUTO_REBALANCE_DECISION.txt</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5398,7 +7241,7 @@
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
@@ -5600,7 +7443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:26</t>
+          <t>2026-06-21T22:54:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5610,12 +7453,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DEFENSE_040838</t>
+          <t>VALMAX_046612</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5626,25 +7469,25 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="M2" t="b">
         <v>0</v>
@@ -5656,7 +7499,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:26</t>
+          <t>2026-06-21T22:54:59</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5676,17 +7519,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I3" t="n">
         <v>10</v>
       </c>
       <c r="J3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="M3" t="b">
         <v>0</v>
@@ -5732,7 +7575,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-20T07:26:26</t>
+          <t>2026-06-21T22:54:59</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5777,183 +7620,4 @@
   <autoFilter ref="A1:AG4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="44" customWidth="1" min="15" max="15"/>
-    <col width="44" customWidth="1" min="16" max="16"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>started_at</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>finished_at</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>lookback_days</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>chunk_size</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>sleep_seconds</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>timeout</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>retry_attempts</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>retry_sleep_seconds</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>updated_symbols</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>updated_symbol_count</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>current_price_rows</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>markets</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="b">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>updated</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>yfinance_target_only</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-06-20T07:26:26</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-06-20T07:26:37</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>30</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>12</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>['TW:2327.TW', 'TW:2454.TW', 'TW:3189.TW', 'US:ARM', 'US:MRVL', 'US:SNDK', 'US:WDC']</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>7</v>
-      </c>
-      <c r="N2" t="n">
-        <v>7</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>[{'market': 'TW', 'status': 'updated', 'start': '2026-05-30', 'symbols': ['2327.TW', '2454.TW', '3189.TW'], 'attempted_symbols': 3, 'chunks_attempted': 3, 'download_attempts': 3, 'retry_attempts': 1, 'retry_sleep_seconds': 12.0, 'updated_symbols': 3, 'skipped_older': [], 'errors': []}, {'market': 'US', 'status': 'updated', 'start': '2026-05-30', 'symbols': ['ARM', 'MRVL', 'SNDK', 'WDC'], 'attempted_symbols': 4, 'chunks_attempted': 4, 'download_attempts': 4, 'retry_attempts': 1, 'retry_sleep_seconds': 12.0, 'updated_symbols': 4, 'skipped_older': [], 'errors': []}]</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Target-only quote refresh updates state/current_prices.csv and entry judgment only. It does not update the full scan pool or retrain strategy rules.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:P2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Switch TW production to fusion H46
</commit_message>
<xml_diff>
--- a/runtime_outputs/DAILY_MARKET_RECORD.xlsx
+++ b/runtime_outputs/DAILY_MARKET_RECORD.xlsx
@@ -20,14 +20,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Today_Order_Plan'!$A$1:$AI$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Order_History'!$A$1:$W$194</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market_State'!$A$1:$AM$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Order_History'!$A$1:$W$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Market_State'!$A$1:$AT$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Target_Position'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Current_Prices'!$A$1:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Current_Holdings'!$A$1:$A$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Update_Report'!$A$1:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Auto_Rebalance'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Summary'!$A$1:$AG$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Summary'!$A$1:$AI$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Target_Price_Refresh'!$A$1:$P$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <col width="19" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
@@ -690,10 +690,10 @@
         <v>1080</v>
       </c>
       <c r="G2" t="n">
-        <v>1080</v>
+        <v>1065</v>
       </c>
       <c r="H2" t="n">
-        <v>1080</v>
+        <v>1065</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -714,13 +714,13 @@
         <v>1000000</v>
       </c>
       <c r="P2" t="n">
-        <v>925</v>
+        <v>938</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>925</v>
+        <v>938</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>-1.388888888888884</v>
       </c>
       <c r="V2" t="n">
-        <v>1080</v>
+        <v>1065</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -767,7 +767,7 @@
         <v>1080</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>-1.388888888888884</v>
       </c>
       <c r="AF2" t="n">
         <v>-7</v>
@@ -1393,12 +1393,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:43</t>
+          <t>2026-06-22T09:49:20</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:57</t>
+          <t>2026-06-22T09:49:36</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>[{'market': 'TW', 'status': 'updated', 'start': '2026-05-31', 'symbols': ['2327.TW'], 'attempted_symbols': 1, 'chunks_attempted': 1, 'download_attempts': 1, 'retry_attempts': 2, 'retry_sleep_seconds': 12.0, 'updated_symbols': 1, 'skipped_older': [], 'errors': []}, {'market': 'US', 'status': 'updated', 'start': '2026-05-31', 'symbols': ['ARM', 'MRVL', 'SNDK', 'WDC'], 'attempted_symbols': 4, 'chunks_attempted': 4, 'download_attempts': 4, 'retry_attempts': 2, 'retry_sleep_seconds': 12.0, 'updated_symbols': 4, 'skipped_older': [], 'errors': []}]</t>
+          <t>[{'market': 'TW', 'status': 'updated', 'start': '2026-06-01', 'symbols': ['2327.TW'], 'attempted_symbols': 1, 'chunks_attempted': 1, 'download_attempts': 1, 'retry_attempts': 2, 'retry_sleep_seconds': 12.0, 'updated_symbols': 1, 'skipped_older': [], 'errors': []}, {'market': 'US', 'status': 'updated', 'start': '2026-06-01', 'symbols': ['ARM', 'MRVL', 'SNDK', 'WDC'], 'attempted_symbols': 4, 'chunks_attempted': 4, 'download_attempts': 4, 'retry_attempts': 2, 'retry_sleep_seconds': 12.0, 'updated_symbols': 4, 'skipped_older': [], 'errors': []}]</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W194"/>
+  <dimension ref="A1:W199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -19547,8 +19547,473 @@
         <v>0</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:20</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:43</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>2327.TW</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>國巨*</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>passive_component</t>
+        </is>
+      </c>
+      <c r="G195" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J195" t="n">
+        <v>938</v>
+      </c>
+      <c r="K195" t="n">
+        <v>0</v>
+      </c>
+      <c r="L195" t="n">
+        <v>938</v>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O195" t="n">
+        <v>-1.388888888888884</v>
+      </c>
+      <c r="P195" t="n">
+        <v>1065</v>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R195" t="n">
+        <v>1080</v>
+      </c>
+      <c r="S195" t="n">
+        <v>1004.4</v>
+      </c>
+      <c r="T195" t="n">
+        <v>1112.4</v>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V195" t="n">
+        <v>1080</v>
+      </c>
+      <c r="W195" t="n">
+        <v>-1.388888888888884</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:20</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:43</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Sandisk Corporation - Common Stock When-Issued</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>memory_storage</t>
+        </is>
+      </c>
+      <c r="G196" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J196" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="K196" t="n">
+        <v>0</v>
+      </c>
+      <c r="L196" t="n">
+        <v>11.44295686005264</v>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O196" t="n">
+        <v>0</v>
+      </c>
+      <c r="P196" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R196" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="S196" t="n">
+        <v>2075.5125</v>
+      </c>
+      <c r="T196" t="n">
+        <v>2293.9875</v>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V196" t="n">
+        <v>2184.75</v>
+      </c>
+      <c r="W196" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:20</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:43</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Arm Holdings plc - American Depositary Shares</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>ai_compute</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J197" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="K197" t="n">
+        <v>0</v>
+      </c>
+      <c r="L197" t="n">
+        <v>56.88800001388867</v>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O197" t="n">
+        <v>0</v>
+      </c>
+      <c r="P197" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R197" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="S197" t="n">
+        <v>417.4869918823242</v>
+      </c>
+      <c r="T197" t="n">
+        <v>461.432991027832</v>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V197" t="n">
+        <v>439.4599914550781</v>
+      </c>
+      <c r="W197" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:20</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:43</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Marvell Technology, Inc. - Common Stock</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>ai_compute</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J198" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="K198" t="n">
+        <v>0</v>
+      </c>
+      <c r="L198" t="n">
+        <v>80.49456204797346</v>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O198" t="n">
+        <v>0</v>
+      </c>
+      <c r="P198" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R198" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="S198" t="n">
+        <v>295.0509872436523</v>
+      </c>
+      <c r="T198" t="n">
+        <v>326.1089859008789</v>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V198" t="n">
+        <v>310.5799865722656</v>
+      </c>
+      <c r="W198" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:20</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-06-22T09:49:43</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Western Digital Corporation - Common Stock</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>memory_storage</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>25000</v>
+      </c>
+      <c r="J199" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="K199" t="n">
+        <v>0</v>
+      </c>
+      <c r="L199" t="n">
+        <v>33.50173626674187</v>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>新增</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>可買滿</t>
+        </is>
+      </c>
+      <c r="O199" t="n">
+        <v>0</v>
+      </c>
+      <c r="P199" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="R199" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="S199" t="n">
+        <v>708.9184814453125</v>
+      </c>
+      <c r="T199" t="n">
+        <v>783.5414794921875</v>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V199" t="n">
+        <v>746.22998046875</v>
+      </c>
+      <c r="W199" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W194"/>
+  <autoFilter ref="A1:W199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19559,48 +20024,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM4"/>
+  <dimension ref="A1:AT4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="29" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="27" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="32" customWidth="1" min="19" max="19"/>
-    <col width="39" customWidth="1" min="20" max="20"/>
-    <col width="23" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="44" customWidth="1" min="23" max="23"/>
-    <col width="35" customWidth="1" min="24" max="24"/>
-    <col width="27" customWidth="1" min="25" max="25"/>
-    <col width="31" customWidth="1" min="26" max="26"/>
-    <col width="26" customWidth="1" min="27" max="27"/>
-    <col width="17" customWidth="1" min="28" max="28"/>
-    <col width="10" customWidth="1" min="29" max="29"/>
-    <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="23" customWidth="1" min="31" max="31"/>
-    <col width="44" customWidth="1" min="32" max="32"/>
-    <col width="27" customWidth="1" min="33" max="33"/>
-    <col width="11" customWidth="1" min="34" max="34"/>
-    <col width="16" customWidth="1" min="35" max="35"/>
-    <col width="34" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
-    <col width="31" customWidth="1" min="38" max="38"/>
-    <col width="31" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="29" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="27" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="32" customWidth="1" min="26" max="26"/>
+    <col width="39" customWidth="1" min="27" max="27"/>
+    <col width="23" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
+    <col width="44" customWidth="1" min="30" max="30"/>
+    <col width="35" customWidth="1" min="31" max="31"/>
+    <col width="27" customWidth="1" min="32" max="32"/>
+    <col width="31" customWidth="1" min="33" max="33"/>
+    <col width="26" customWidth="1" min="34" max="34"/>
+    <col width="17" customWidth="1" min="35" max="35"/>
+    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="37" max="37"/>
+    <col width="23" customWidth="1" min="38" max="38"/>
+    <col width="44" customWidth="1" min="39" max="39"/>
+    <col width="27" customWidth="1" min="40" max="40"/>
+    <col width="11" customWidth="1" min="41" max="41"/>
+    <col width="16" customWidth="1" min="42" max="42"/>
+    <col width="34" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="31" customWidth="1" min="45" max="45"/>
+    <col width="31" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19661,140 +20133,175 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>selected_sleeve</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>component_signal_date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>component_rebalance_date</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>component_top_score</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>component_second_score</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>attack_score</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>recommend_score</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>attack_edge</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>attack_dd60</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>attack_r60</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>rebalance_step_trading_days</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>trading_days_since_rebalance</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>trading_days_since_signal</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>rebalance_days_remaining</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>rebalance_due_today_by_counter</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>rebalance_due_next_session_by_counter</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>rebalance_count_basis</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>action_signal</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>research_component_rebalance_date</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>live_cycle_rebalance_date</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>live_cycle_source_signal_date</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>live_cycle_baseline_type</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>execution_top_n</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>regime</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>gross_cap</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>scan_universe_symbols</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>dynamic_market_pool</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>uses_2025_2026_for_tuning</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>top_stock</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>top_theme</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>outside_execution_count_in_top20</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>watch_only</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>feeds_dynamic_market_strategy</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>feeds_dynamic_formal_strategy</t>
         </is>
@@ -19813,12 +20320,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:37</t>
+          <t>2026-06-22T09:49:15</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TW_TOP1_TOP2_SWITCH_H46_TH020_CLEAN</t>
+          <t>TW_ATTACK_RECOMMEND_FUSION_H46_EDGE005_CLEAN</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -19828,7 +20335,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>top1_top2_switch_h46_th020</t>
+          <t>attack_recommend_fusion_h46_edge005</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -19844,7 +20351,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>top1_top2_switch_h46_th020</t>
+          <t>attack_recommend_fusion_h46_edge005</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -19854,7 +20361,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -19862,58 +20369,81 @@
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>0.6451507360937982</v>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
       </c>
       <c r="O2" t="n">
+        <v>0.5209533492052429</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.4900682791335889</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.455748008895623</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.3073196089363748</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.1484283999592482</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.5274669881598333</v>
+      </c>
+      <c r="V2" t="n">
         <v>46</v>
       </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
         <v>46</v>
       </c>
-      <c r="S2" t="b">
-        <v>0</v>
-      </c>
-      <c r="T2" t="b">
-        <v>0</v>
-      </c>
-      <c r="U2" t="inlineStr">
+      <c r="Z2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>live_go_live_cycle</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>hold_live_cycle_target</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>TW production target uses clean Top1/Top2 Switch H46 threshold 0.20, then applies execution overlay: equal weight across selected stocks. Manual go-live baseline recomputes the initial live target from that baseline close and then holds it until the next live cycle. No retraining in cloud package. Live cycle starts from 2026-06-18 because formal deployment was reset manually.</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>TW production target uses clean Attack/Recommend Fusion H46. Attack sleeve is used only when its sleeve score beats recommend by 0.05, attack 60D return is non-negative, and attack 60D drawdown stays above -60%; otherwise recommend sleeve is used. Execution overlay remains equal weight across selected stocks. Manual go-live baseline recomputes the initial live target from that baseline close and then holds it until the next live cycle. No retraining in cloud package. Live cycle starts from 2026-06-18 because formal deployment was reset manually.</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>manual_go_live_close</t>
         </is>
@@ -19932,7 +20462,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:42</t>
+          <t>2026-06-22T09:49:19</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -19955,84 +20485,84 @@
           <t>TOP5_R800_N5_COMBO</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
         <v>0.7553501447582477</v>
       </c>
-      <c r="O3" t="n">
+      <c r="V3" t="n">
         <v>10</v>
       </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>10</v>
       </c>
-      <c r="S3" t="b">
-        <v>0</v>
-      </c>
-      <c r="T3" t="b">
-        <v>0</v>
-      </c>
-      <c r="U3" t="inlineStr">
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
         <is>
           <t>live_go_live_cycle</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>US production target uses the clean dynamic-market switch with Top4 execution and 25% single-stock cap. Rules are frozen; no cloud retraining. Live cycle starts from 2026-06-18 because formal deployment was reset manually.</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>2026-06-10</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
         <is>
           <t>manual_go_live_close</t>
         </is>
       </c>
-      <c r="AB3" t="n">
+      <c r="AI3" t="n">
         <v>4</v>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>risk_on</t>
         </is>
       </c>
-      <c r="AD3" t="n">
+      <c r="AK3" t="n">
         <v>1</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AL3" t="n">
         <v>812</v>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>rolling Top800 by 60D median dollar volume</t>
         </is>
       </c>
-      <c r="AG3" t="b">
+      <c r="AN3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -20049,37 +20579,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:43</t>
-        </is>
-      </c>
-      <c r="AE4" t="n">
+          <t>2026-06-22T09:49:20</t>
+        </is>
+      </c>
+      <c r="AL4" t="n">
         <v>812</v>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AO4" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AP4" t="inlineStr">
         <is>
           <t>memory_storage</t>
         </is>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AQ4" t="n">
         <v>11</v>
       </c>
-      <c r="AK4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL4" t="b">
+      <c r="AR4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="b">
         <v>1</v>
       </c>
-      <c r="AM4" t="b">
+      <c r="AT4" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM4"/>
+  <autoFilter ref="A1:AT4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20186,7 +20716,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>top1_top2_switch_DEFENSE_040838__TOP1|equal_weight_exec</t>
+          <t>tw_fusion_attack_DEFENSE_040838__TOP1|equal_weight_exec</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -20430,11 +20960,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1080</v>
+        <v>1065</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -20444,7 +20974,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:49</t>
+          <t>2026-06-22T09:49:27</t>
         </is>
       </c>
     </row>
@@ -20534,7 +21064,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:51</t>
+          <t>2026-06-22T09:49:29</t>
         </is>
       </c>
     </row>
@@ -20564,7 +21094,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:53</t>
+          <t>2026-06-22T09:49:32</t>
         </is>
       </c>
     </row>
@@ -20594,7 +21124,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:55</t>
+          <t>2026-06-22T09:49:34</t>
         </is>
       </c>
     </row>
@@ -20624,7 +21154,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:57</t>
+          <t>2026-06-22T09:49:36</t>
         </is>
       </c>
     </row>
@@ -21296,7 +21826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -21305,33 +21835,35 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="29" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="37" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
     <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="32" customWidth="1" min="13" max="13"/>
-    <col width="39" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="29" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="44" customWidth="1" min="21" max="21"/>
-    <col width="23" customWidth="1" min="22" max="22"/>
-    <col width="28" customWidth="1" min="23" max="23"/>
-    <col width="28" customWidth="1" min="24" max="24"/>
-    <col width="23" customWidth="1" min="25" max="25"/>
-    <col width="34" customWidth="1" min="26" max="26"/>
-    <col width="27" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
-    <col width="34" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="31" customWidth="1" min="32" max="32"/>
-    <col width="44" customWidth="1" min="33" max="33"/>
+    <col width="29" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="39" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="44" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="24" max="24"/>
+    <col width="28" customWidth="1" min="25" max="25"/>
+    <col width="28" customWidth="1" min="26" max="26"/>
+    <col width="23" customWidth="1" min="27" max="27"/>
+    <col width="34" customWidth="1" min="28" max="28"/>
+    <col width="27" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="34" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="31" customWidth="1" min="34" max="34"/>
+    <col width="44" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21367,135 +21899,145 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>strategy_mode</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>selected_sleeve</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>selected_component</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>attack_edge</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>component_signal_date</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>component_rebalance_date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>rebalance_step_trading_days</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>trading_days_since_rebalance</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>trading_days_since_signal</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rebalance_days_remaining</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>rebalance_due_today_by_counter</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>rebalance_due_next_session_by_counter</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>regime</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>gross_cap</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>strategy_mode</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>execution_overlay</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>execution_top_n</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>selected_component</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>dynamic_market_pool</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>scan_universe_symbols</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>dynamic_formal_gate_active</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>dynamic_formal_gate_reason</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>dynamic_formal_weight</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>dynamic_formal_latest_price_date</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>dynamic_formal_pool_count</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>top_stock</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>top_theme</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>outside_execution_count_in_top20</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>watch_only</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>feeds_dynamic_market_strategy</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -21504,7 +22046,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:43</t>
+          <t>2026-06-22T09:49:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -21530,37 +22072,55 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>attack_recommend_fusion_h46_edge005</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
+          <t>attack</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>DEFENSE_040838__TOP1</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0.1484283999592482</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>46</v>
       </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
         <v>46</v>
       </c>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N2" t="b">
+      <c r="Q2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:43</t>
+          <t>2026-06-22T09:49:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -21575,68 +22135,68 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>top1_dynamic_market_like_tw</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>TOP5_R800_N5_COMBO</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>10</v>
       </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
         <v>10</v>
       </c>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
-      <c r="N3" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>risk_on</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="T3" t="n">
         <v>1</v>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>top1_dynamic_market_like_tw</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>US_DYNAMIC_MARKET_TOP4_CAP25</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="V3" t="n">
         <v>4</v>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>TOP5_R800_N5_COMBO</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>rolling Top800 by 60D median dollar volume</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>812</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-21T23:56:43</t>
+          <t>2026-06-22T09:49:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -21649,36 +22209,36 @@
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>812</v>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>memory_storage</t>
         </is>
       </c>
-      <c r="AD4" t="n">
+      <c r="AF4" t="n">
         <v>11</v>
       </c>
-      <c r="AE4" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF4" t="b">
+      <c r="AG4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="b">
         <v>1</v>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>US_SCAN monitors the rolling Top800 market pool. The official US Top1 dynamic-market strategy can select from this live pool when frozen rules pass.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG4"/>
+  <autoFilter ref="A1:AI4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>